<commit_message>
feat: adding knowledge database to ai
</commit_message>
<xml_diff>
--- a/base.xlsx
+++ b/base.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mauricio.santos\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mauricio.santos\Desktop\gruposc.ia\sup sistemas ia\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="103">
   <si>
     <t>processo</t>
   </si>
@@ -312,7 +312,32 @@
     <t>descricao</t>
   </si>
   <si>
-    <t>Emissão de NFI (Nota Fiscal de Incineração)</t>
+    <t>Classificação e determinação de NFOs</t>
+  </si>
+  <si>
+    <t>Monitor de compras, onde é gerado a id agrupamento</t>
+  </si>
+  <si>
+    <t>Monitor fiscal para Ids, onde é gerado o espelho para emissão da NFD</t>
+  </si>
+  <si>
+    <t>101 - avaria interna
+102 - avaria externa
+108 - avaria Cross
+013 - avaria fob
+113 - avaria comercial</t>
+  </si>
+  <si>
+    <t>explicacao</t>
+  </si>
+  <si>
+    <t>depositos</t>
+  </si>
+  <si>
+    <t>Emissão de NF Devolução (NFD)</t>
+  </si>
+  <si>
+    <t>Emissão de NF de Incineração (NFI)</t>
   </si>
 </sst>
 </file>
@@ -348,8 +373,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -630,15 +658,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.26953125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="35.54296875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="60" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>93</v>
       </c>
@@ -648,8 +677,11 @@
       <c r="C1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -660,7 +692,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -670,8 +702,11 @@
       <c r="C3" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -682,7 +717,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -693,7 +728,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -704,7 +739,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -715,7 +750,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -726,7 +761,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -737,7 +772,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -748,7 +783,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -759,7 +794,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -770,7 +805,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -781,7 +816,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -792,7 +827,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>25</v>
       </c>
@@ -803,7 +838,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>27</v>
       </c>
@@ -814,7 +849,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -825,7 +860,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>31</v>
       </c>
@@ -836,7 +871,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>33</v>
       </c>
@@ -847,7 +882,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>35</v>
       </c>
@@ -858,7 +893,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>37</v>
       </c>
@@ -868,8 +903,11 @@
       <c r="C21" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D21" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>39</v>
       </c>
@@ -879,8 +917,11 @@
       <c r="C22" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D22" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>41</v>
       </c>
@@ -890,8 +931,11 @@
       <c r="C23" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D23" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>43</v>
       </c>
@@ -902,7 +946,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>45</v>
       </c>
@@ -913,7 +957,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>47</v>
       </c>
@@ -924,7 +968,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>49</v>
       </c>
@@ -935,7 +979,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>51</v>
       </c>
@@ -946,7 +990,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>53</v>
       </c>
@@ -957,7 +1001,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>55</v>
       </c>
@@ -968,7 +1012,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>57</v>
       </c>
@@ -979,7 +1023,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>59</v>
       </c>
@@ -990,7 +1034,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>61</v>
       </c>
@@ -1001,7 +1045,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>63</v>
       </c>
@@ -1012,7 +1056,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>65</v>
       </c>
@@ -1023,7 +1067,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>67</v>
       </c>
@@ -1034,7 +1078,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>69</v>
       </c>
@@ -1045,7 +1089,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>71</v>
       </c>
@@ -1056,7 +1100,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>73</v>
       </c>
@@ -1067,7 +1111,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>75</v>
       </c>
@@ -1078,7 +1122,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>77</v>
       </c>
@@ -1089,7 +1133,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>80</v>
       </c>
@@ -1100,7 +1144,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>82</v>
       </c>
@@ -1110,8 +1154,11 @@
       <c r="C43" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D43" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>84</v>
       </c>
@@ -1122,7 +1169,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>86</v>
       </c>
@@ -1133,7 +1180,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>88</v>
       </c>
@@ -1144,7 +1191,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>90</v>
       </c>
@@ -1162,15 +1209,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.08984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="37.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>93</v>
       </c>
@@ -1180,8 +1229,14 @@
       <c r="C1" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>86</v>
       </c>
@@ -1189,7 +1244,21 @@
         <v>87</v>
       </c>
       <c r="C2" t="s">
-        <v>95</v>
+        <v>102</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: front end ajust
</commit_message>
<xml_diff>
--- a/base.xlsx
+++ b/base.xlsx
@@ -9,11 +9,12 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6640"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6640" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="geral" sheetId="1" r:id="rId1"/>
     <sheet name="segregados" sheetId="2" r:id="rId2"/>
+    <sheet name="erros" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="106">
   <si>
     <t>processo</t>
   </si>
@@ -335,6 +336,18 @@
   </si>
   <si>
     <t>Emissão de NF de Incineração (NFI)</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>DEV01</t>
+  </si>
+  <si>
+    <t>Saldo não é igual a zero: xxx,xx débito: xxx,xx Crédito: xxx,xx</t>
+  </si>
+  <si>
+    <t>erro</t>
   </si>
 </sst>
 </file>
@@ -1250,4 +1263,34 @@
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="51.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
build: ajust prompt ai
</commit_message>
<xml_diff>
--- a/base.xlsx
+++ b/base.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6640" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6640"/>
   </bookViews>
   <sheets>
     <sheet name="geral" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="110">
   <si>
     <t>processo</t>
   </si>
@@ -348,6 +348,18 @@
   </si>
   <si>
     <t>erro</t>
+  </si>
+  <si>
+    <t>MI31</t>
+  </si>
+  <si>
+    <t>Batch Input: criar doc.invent.</t>
+  </si>
+  <si>
+    <t>inventario</t>
+  </si>
+  <si>
+    <t>criação de documento de inventário</t>
   </si>
 </sst>
 </file>
@@ -668,7 +680,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.26953125" bestFit="1" customWidth="1"/>
@@ -1199,6 +1211,20 @@
       </c>
       <c r="C46" t="s">
         <v>78</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>106</v>
+      </c>
+      <c r="B47" t="s">
+        <v>107</v>
+      </c>
+      <c r="C47" t="s">
+        <v>108</v>
+      </c>
+      <c r="D47" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>